<commit_message>
feat: add example files
</commit_message>
<xml_diff>
--- a/excel/Hero/hero.xlsx
+++ b/excel/Hero/hero.xlsx
@@ -4,11 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="18980" activeTab="1"/>
+    <workbookView windowHeight="18980"/>
   </bookViews>
   <sheets>
-    <sheet name="hero" sheetId="1" r:id="rId1"/>
-    <sheet name="conf" sheetId="2" r:id="rId2"/>
+    <sheet name="Base" sheetId="1" r:id="rId1"/>
+    <sheet name="Level" sheetId="7" r:id="rId2"/>
+    <sheet name="Skill" sheetId="8" r:id="rId3"/>
+    <sheet name="Constant" sheetId="9" r:id="rId4"/>
+    <sheet name="_metadata" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,9 +31,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
-  <si>
-    <t>table</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="72">
+  <si>
+    <t>table_base</t>
   </si>
   <si>
     <t>Hero ID</t>
@@ -39,6 +42,18 @@
     <t>Hero Name</t>
   </si>
   <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Quality</t>
+  </si>
+  <si>
+    <t>Pieces To Unlock Hero</t>
+  </si>
+  <si>
     <t>name</t>
   </si>
   <si>
@@ -48,9 +63,33 @@
     <t>Name</t>
   </si>
   <si>
+    <t>Joined#HeroLevel_Level</t>
+  </si>
+  <si>
+    <t>JoinedList#HeroSkill_Skill</t>
+  </si>
+  <si>
+    <t>QualityInt</t>
+  </si>
+  <si>
+    <t>Type#Costs_Cost</t>
+  </si>
+  <si>
     <t>proto</t>
   </si>
   <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Skill</t>
+  </si>
+  <si>
+    <t>Pieces</t>
+  </si>
+  <si>
+    <t>condition</t>
+  </si>
+  <si>
     <t>type</t>
   </si>
   <si>
@@ -60,10 +99,142 @@
     <t>string</t>
   </si>
   <si>
+    <t>[]int</t>
+  </si>
+  <si>
+    <t>uint</t>
+  </si>
+  <si>
+    <t>map[int]uint</t>
+  </si>
+  <si>
     <t>Monkey D.Luffy</t>
   </si>
   <si>
+    <t>101#102</t>
+  </si>
+  <si>
+    <t>4$1</t>
+  </si>
+  <si>
     <t>Roronoa Zoro</t>
+  </si>
+  <si>
+    <t>201#202</t>
+  </si>
+  <si>
+    <t>5$6</t>
+  </si>
+  <si>
+    <t>table_level</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Hero Level Atk</t>
+  </si>
+  <si>
+    <t>Hero Level Hp</t>
+  </si>
+  <si>
+    <t>required to upgrade to this level</t>
+  </si>
+  <si>
+    <t>prizes when upgraded</t>
+  </si>
+  <si>
+    <t>SharedId_Id</t>
+  </si>
+  <si>
+    <t>SharedSubId_Level</t>
+  </si>
+  <si>
+    <t>Atk</t>
+  </si>
+  <si>
+    <t>Hp</t>
+  </si>
+  <si>
+    <t>Type#PackPrizes_Prize</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Prize</t>
+  </si>
+  <si>
+    <t>Level 1</t>
+  </si>
+  <si>
+    <t>Level 2</t>
+  </si>
+  <si>
+    <t>4$2#3$20</t>
+  </si>
+  <si>
+    <t>1$1</t>
+  </si>
+  <si>
+    <t>Level 3</t>
+  </si>
+  <si>
+    <t>4$5#3$50</t>
+  </si>
+  <si>
+    <t>1$2</t>
+  </si>
+  <si>
+    <t>table_skill</t>
+  </si>
+  <si>
+    <t>Shared_Name</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>Gomu Gomu Rocket</t>
+  </si>
+  <si>
+    <t>Gomu Gomu Snake Gun</t>
+  </si>
+  <si>
+    <t>Purgatory Demon Slash</t>
+  </si>
+  <si>
+    <t>Ashura Makyusen</t>
+  </si>
+  <si>
+    <t>kv_constant</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Client Field</t>
+  </si>
+  <si>
+    <t>Condition</t>
+  </si>
+  <si>
+    <t>Value Type</t>
+  </si>
+  <si>
+    <t>ClientField</t>
+  </si>
+  <si>
+    <t>ValueType</t>
+  </si>
+  <si>
+    <t>Heroes on created</t>
+  </si>
+  <si>
+    <t>JoinedList#HeroBase_Hero</t>
   </si>
   <si>
     <t>key</t>
@@ -88,9 +259,16 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -105,21 +283,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="微软雅黑"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="微软雅黑"/>
       <charset val="134"/>
@@ -493,7 +671,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -517,6 +695,19 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color theme="0" tint="-0.149143955809198"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.149143955809198"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.149143955809198"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color rgb="FFDEE0E3"/>
       </left>
@@ -526,6 +717,36 @@
       <top/>
       <bottom style="medium">
         <color rgb="FFDEE0E3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.149143955809198"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.149143955809198"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.149143955809198"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.149143955809198"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.149113437299722"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.149113437299722"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.149113437299722"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.149113437299722"/>
       </bottom>
       <diagonal/>
     </border>
@@ -643,7 +864,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
@@ -662,175 +883,215 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="51">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
     <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
     <cellStyle name="货币" xfId="2" builtinId="4"/>
@@ -880,6 +1141,8 @@
     <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
     <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+    <cellStyle name="常规 5" xfId="49"/>
+    <cellStyle name="常规 2" xfId="50"/>
   </cellStyles>
   <dxfs count="18">
     <dxf>
@@ -1364,78 +1627,181 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="5" outlineLevelCol="2"/>
+  <dimension ref="A1:T7"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="6"/>
   <cols>
-    <col min="1" max="1" width="14.6153846153846" style="4" customWidth="1"/>
-    <col min="2" max="2" width="14.8942307692308" style="4" customWidth="1"/>
-    <col min="3" max="3" width="25" style="4" customWidth="1"/>
+    <col min="1" max="1" width="14.6153846153846" style="20" customWidth="1"/>
+    <col min="2" max="2" width="14.8942307692308" style="21" customWidth="1"/>
+    <col min="3" max="3" width="25" style="21" customWidth="1"/>
+    <col min="4" max="4" width="35.0961538461538" style="21" customWidth="1"/>
+    <col min="5" max="5" width="30.0769230769231" style="21" customWidth="1"/>
+    <col min="6" max="6" width="12.9807692307692" style="21" customWidth="1"/>
+    <col min="7" max="7" width="27.0769230769231" style="21" customWidth="1"/>
+    <col min="8" max="16384" width="9.23076923076923" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.6" spans="1:3">
-      <c r="A1" s="5" t="s">
+    <row r="1" s="8" customFormat="1" ht="17.6" spans="1:7">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" ht="17.6" spans="1:3">
-      <c r="A2" s="7" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" ht="17.6" spans="1:3">
-      <c r="A3" s="7" t="s">
+      <c r="G1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="8" t="s">
+    </row>
+    <row r="2" s="11" customFormat="1" ht="17.6" spans="1:7">
+      <c r="A2" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" s="11" customFormat="1" ht="17.6" spans="1:7">
+      <c r="A3" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="11" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" ht="17.6" spans="1:3">
-      <c r="A4" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" ht="18.35" spans="1:3">
-      <c r="A5" s="11"/>
-      <c r="B5" s="12">
+      <c r="G3" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" s="11" customFormat="1" ht="17.6" spans="1:3">
+      <c r="A4" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+    </row>
+    <row r="5" s="13" customFormat="1" ht="17.6" spans="1:7">
+      <c r="A5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" s="15" customFormat="1" ht="18.35" spans="1:20">
+      <c r="A6" s="14"/>
+      <c r="B6" s="16">
         <v>1</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" ht="18.35" spans="1:3">
-      <c r="A6" s="11"/>
-      <c r="B6" s="13">
+      <c r="C6" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="16">
+        <v>1</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="16">
+        <v>5</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
+      <c r="P6" s="16"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="16"/>
+      <c r="S6" s="16"/>
+      <c r="T6" s="16"/>
+    </row>
+    <row r="7" s="17" customFormat="1" ht="18.35" spans="1:13">
+      <c r="A7" s="14"/>
+      <c r="B7" s="23">
         <v>2</v>
       </c>
-      <c r="C6" s="13" t="s">
-        <v>11</v>
-      </c>
+      <c r="C7" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="23">
+        <v>1</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="23">
+        <v>5</v>
+      </c>
+      <c r="G7" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B5:B6">
+  <conditionalFormatting sqref="B6:B7">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1446,27 +1812,626 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="1" outlineLevelCol="1"/>
+  <dimension ref="A1:R8"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="7"/>
   <cols>
-    <col min="1" max="1" width="14.6923076923077" customWidth="1"/>
+    <col min="1" max="1" width="14.6153846153846" style="20" customWidth="1"/>
+    <col min="2" max="2" width="14.8942307692308" style="21" customWidth="1"/>
+    <col min="3" max="3" width="24.9230769230769" style="21" customWidth="1"/>
+    <col min="4" max="4" width="25" style="21" customWidth="1"/>
+    <col min="5" max="5" width="17.7692307692308" style="21" customWidth="1"/>
+    <col min="6" max="6" width="17.3076923076923" style="21" customWidth="1"/>
+    <col min="7" max="7" width="39.3076923076923" style="21" customWidth="1"/>
+    <col min="8" max="8" width="27.5384615384615" style="21" customWidth="1"/>
+    <col min="9" max="16384" width="9.23076923076923" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.6" spans="1:2">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="8" customFormat="1" ht="17.6" spans="1:8">
+      <c r="A1" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" s="11" customFormat="1" ht="17.6" spans="1:8">
+      <c r="A2" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" s="11" customFormat="1" ht="17.6" spans="1:8">
+      <c r="A3" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" s="11" customFormat="1" ht="17.6" spans="1:4">
+      <c r="A4" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+    </row>
+    <row r="5" s="13" customFormat="1" ht="17.6" spans="1:8">
+      <c r="A5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" s="15" customFormat="1" ht="18.35" spans="1:18">
+      <c r="A6" s="14"/>
+      <c r="B6" s="16">
+        <v>1</v>
+      </c>
+      <c r="C6" s="16">
+        <v>1</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="16">
+        <v>20</v>
+      </c>
+      <c r="F6" s="16">
+        <v>600</v>
+      </c>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
+      <c r="P6" s="16"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="16"/>
+    </row>
+    <row r="7" s="17" customFormat="1" ht="18.35" spans="1:11">
+      <c r="A7" s="14"/>
+      <c r="B7" s="23">
+        <v>1</v>
+      </c>
+      <c r="C7" s="23">
+        <v>2</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="23">
+        <v>40</v>
+      </c>
+      <c r="F7" s="23">
+        <v>1000</v>
+      </c>
+      <c r="G7" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="H7" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+    </row>
+    <row r="8" s="18" customFormat="1" ht="18.35" spans="1:18">
+      <c r="A8" s="14"/>
+      <c r="B8" s="23">
+        <v>1</v>
+      </c>
+      <c r="C8" s="24">
+        <v>3</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="17">
+        <v>60</v>
+      </c>
+      <c r="F8" s="17">
+        <v>1600</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
+      <c r="N8" s="20"/>
+      <c r="O8" s="20"/>
+      <c r="P8" s="20"/>
+      <c r="Q8" s="20"/>
+      <c r="R8" s="20"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B6:C8">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:S11"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8"/>
+  <cols>
+    <col min="1" max="1" width="14.6153846153846" style="20" customWidth="1"/>
+    <col min="2" max="2" width="15.6923076923077" style="21" customWidth="1"/>
+    <col min="3" max="3" width="29.6923076923077" style="21" customWidth="1"/>
+    <col min="4" max="4" width="35.0961538461538" style="21" customWidth="1"/>
+    <col min="5" max="5" width="20.1826923076923" style="21" customWidth="1"/>
+    <col min="6" max="16384" width="9.23076923076923" style="21"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="8" customFormat="1" ht="17.6" spans="1:5">
+      <c r="A1" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" s="11" customFormat="1" ht="17.6" spans="1:5">
+      <c r="A2" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" s="11" customFormat="1" ht="17.6" spans="1:5">
+      <c r="A3" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" s="11" customFormat="1" ht="17.6" spans="1:3">
+      <c r="A4" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+    </row>
+    <row r="5" s="13" customFormat="1" ht="17.6" spans="1:5">
+      <c r="A5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" s="15" customFormat="1" ht="18.35" spans="1:19">
+      <c r="A6" s="14"/>
+      <c r="B6" s="16">
+        <v>101</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="16">
+        <v>11</v>
+      </c>
+      <c r="E6" s="16">
+        <v>100</v>
+      </c>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
+      <c r="P6" s="16"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="16"/>
+      <c r="S6" s="16"/>
+    </row>
+    <row r="7" s="17" customFormat="1" ht="18.35" spans="1:19">
+      <c r="A7" s="14"/>
+      <c r="B7" s="23">
+        <v>101</v>
+      </c>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23">
         <v>12</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" ht="17.6" spans="1:2">
-      <c r="A2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="E7" s="23">
+        <v>120</v>
+      </c>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="25"/>
+      <c r="N7" s="25"/>
+      <c r="O7" s="25"/>
+      <c r="P7" s="25"/>
+      <c r="Q7" s="25"/>
+      <c r="R7" s="25"/>
+      <c r="S7" s="25"/>
+    </row>
+    <row r="8" s="17" customFormat="1" ht="18.35" spans="1:12">
+      <c r="A8" s="14"/>
+      <c r="B8" s="23">
+        <v>102</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="23">
+        <v>1</v>
+      </c>
+      <c r="E8" s="23">
+        <v>200</v>
+      </c>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="23"/>
+    </row>
+    <row r="9" s="18" customFormat="1" ht="18.35" spans="1:19">
+      <c r="A9" s="14"/>
+      <c r="B9" s="23">
+        <v>201</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="23">
+        <v>1</v>
+      </c>
+      <c r="E9" s="24">
+        <v>150</v>
+      </c>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="23"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="23"/>
+      <c r="M9" s="20"/>
+      <c r="N9" s="20"/>
+      <c r="O9" s="20"/>
+      <c r="P9" s="20"/>
+      <c r="Q9" s="20"/>
+      <c r="R9" s="20"/>
+      <c r="S9" s="20"/>
+    </row>
+    <row r="10" s="19" customFormat="1" ht="17.55" spans="1:19">
+      <c r="A10" s="20"/>
+      <c r="B10" s="23">
+        <v>202</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="23">
+        <v>1</v>
+      </c>
+      <c r="E10" s="20">
+        <v>180</v>
+      </c>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="20"/>
+      <c r="N10" s="20"/>
+      <c r="O10" s="20"/>
+      <c r="P10" s="20"/>
+      <c r="Q10" s="20"/>
+      <c r="R10" s="20"/>
+      <c r="S10" s="20"/>
+    </row>
+    <row r="11" ht="17.55" spans="2:12">
+      <c r="B11" s="23"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="20"/>
+      <c r="I11" s="20"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B6:B11">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="4" outlineLevelCol="6"/>
+  <cols>
+    <col min="1" max="1" width="15.8461538461538" customWidth="1"/>
+    <col min="2" max="2" width="22.2307692307692" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="13.4615384615385" customWidth="1"/>
+    <col min="5" max="5" width="11.6923076923077" customWidth="1"/>
+    <col min="6" max="6" width="13.4615384615385" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.6" spans="1:7">
+      <c r="A1" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" ht="17.6" spans="1:7">
+      <c r="A2" s="10"/>
+      <c r="B2" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" ht="17.6" spans="1:7">
+      <c r="A3" s="10"/>
+      <c r="B3" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" ht="18.35" spans="1:7">
+      <c r="A4" s="14"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" ht="17.55" spans="1:7">
+      <c r="A5" s="16"/>
+      <c r="B5" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="16">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="17.6" outlineLevelRow="2" outlineLevelCol="1"/>
+  <cols>
+    <col min="1" max="1" width="20.0769230769231" style="3" customWidth="1"/>
+    <col min="2" max="2" width="15.5288461538462" style="2" customWidth="1"/>
+    <col min="3" max="16384" width="9.23076923076923" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" spans="1:2">
+      <c r="A1" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" s="2" customFormat="1" spans="1:2">
+      <c r="A2" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" s="2" customFormat="1" spans="1:2">
+      <c r="A3" s="5"/>
+      <c r="B3" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>